<commit_message>
tested all subdomains of pravartiya
</commit_message>
<xml_diff>
--- a/Pravartiya/data/Searching_agent_output copy.xlsx
+++ b/Pravartiya/data/Searching_agent_output copy.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="106">
   <si>
     <t>Verticals</t>
   </si>
@@ -167,6 +167,171 @@
   </si>
   <si>
     <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/Listed Companies/Circular-NSE/2026/January/Update_on_single_filing_system_through_API_based_integration_between_Stock_Excha_e6aa1e30.pdf</t>
+  </si>
+  <si>
+    <t>April</t>
+  </si>
+  <si>
+    <t>2026-04-30</t>
+  </si>
+  <si>
+    <t>Master Circular for Listed Companies</t>
+  </si>
+  <si>
+    <t>https://nsearchives.nseindia.com//web/circular/2026-04/Master_Circular_NSE_2026.zip</t>
+  </si>
+  <si>
+    <t>Master_Circular_for_Listed_Companies_ed365418.pdf</t>
+  </si>
+  <si>
+    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/Listed Companies/Circular-NSE/2026/April/Master_Circular_for_Listed_Companies_ed365418.pdf</t>
+  </si>
+  <si>
+    <t>2026-04-24</t>
+  </si>
+  <si>
+    <t>Update of single filing system through API-based integration between Stock Exchanges</t>
+  </si>
+  <si>
+    <t>https://nsearchives.nseindia.com//web/circular/2026-04/API_Circular_24_April_2026_20260424200426.pdf</t>
+  </si>
+  <si>
+    <t>Update_of_single_filing_system_through_API_based_integration_between_Stock_Excha_3e21338b.pdf</t>
+  </si>
+  <si>
+    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/Listed Companies/Circular-NSE/2026/April/Update_of_single_filing_system_through_API_based_integration_between_Stock_Excha_3e21338b.pdf</t>
+  </si>
+  <si>
+    <t>2026-04-20</t>
+  </si>
+  <si>
+    <t>https://nsearchives.nseindia.com//web/circular/2026-04/Circular_for_update_on_single_filing_system_through_API-based_integration_between_Stock_Exchanges_20260420201527.pdf</t>
+  </si>
+  <si>
+    <t>Update_of_single_filing_system_through_API_based_integration_between_Stock_Excha_9c408ec3.pdf</t>
+  </si>
+  <si>
+    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/Listed Companies/Circular-NSE/2026/April/Update_of_single_filing_system_through_API_based_integration_between_Stock_Excha_9c408ec3.pdf</t>
+  </si>
+  <si>
+    <t>2026-04-10</t>
+  </si>
+  <si>
+    <t>Ease of doing business - mechanism for lock-in of pledged shares under SEBI (Issue of Capital and Disclosure Requirements) Regulations, 2018</t>
+  </si>
+  <si>
+    <t>https://nsearchives.nseindia.com//web/circular/2026-04/Ease_of_doing_business_mechanism_for_lock-in_of_pledged_shares_under_SEBI_Issue_of_Capital_and_Disclosure_Requirements_Regulations_2018_20260410123152.pdf</t>
+  </si>
+  <si>
+    <t>Ease_of_doing_business_mechanism_for_lock_in_of_pledged_shares_under_SEBI_Issue_8c96f01f.pdf</t>
+  </si>
+  <si>
+    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/Listed Companies/Circular-NSE/2026/April/Ease_of_doing_business_mechanism_for_lock_in_of_pledged_shares_under_SEBI_Issue_8c96f01f.pdf</t>
+  </si>
+  <si>
+    <t>2026-04-07</t>
+  </si>
+  <si>
+    <t>Relaxation from the applicability of SEBI Master Circular for compliance with the provisions of the SEBI (Listing Obligations and Disclosure Requirements) Regulations, 2015 on non-compliance with the Minimum Public Shareholding (MPS) requirements.</t>
+  </si>
+  <si>
+    <t>https://nsearchives.nseindia.com//web/circular/2026-04/MPS_Relaxation_Circular_20260407182420.pdf</t>
+  </si>
+  <si>
+    <t>Relaxation_from_the_applicability_of_SEBI_Master_Circular_for_compliance_with_th_f446a832.pdf</t>
+  </si>
+  <si>
+    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/Listed Companies/Circular-NSE/2026/April/Relaxation_from_the_applicability_of_SEBI_Master_Circular_for_compliance_with_th_f446a832.pdf</t>
+  </si>
+  <si>
+    <t>Informal Guidance</t>
+  </si>
+  <si>
+    <t>February</t>
+  </si>
+  <si>
+    <t>2026-02-06</t>
+  </si>
+  <si>
+    <t>Request for Informal Guidance by way of an interpretative letter under the Securities and Exchange Board of India (Informal Guidance) Scheme, 2025 received from Punjab National Bank seeking interpretation of the provisions of Regulation 27 of the SEBI (Listing Obligations and Disclosure Requirements) Regulations, 2015 and SEBI Circular for implementation of recommendations of the Expert Committee for facilitating ease of doing business for listed entities dated 31.12.2024</t>
+  </si>
+  <si>
+    <t>https://www.sebi.gov.in/sebi_data/commondocs/feb-2026/PNB%20-%20Informal%20Guidance%20Letter%20by%20SEBI_p.pdf</t>
+  </si>
+  <si>
+    <t>Request_for_Informal_Guidance_by_way_of_an_interpretative_letter_under_the_Secur_948a270a.pdf</t>
+  </si>
+  <si>
+    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/SEBI/Informal Guidance/2026/February/Request_for_Informal_Guidance_by_way_of_an_interpretative_letter_under_the_Secur_948a270a.pdf</t>
+  </si>
+  <si>
+    <t>Circular-BSE</t>
+  </si>
+  <si>
+    <t>2026-02-20</t>
+  </si>
+  <si>
+    <t>https://www.bseindia.com/markets/MarketInfo/DispNewNoticesCirculars?page=20260220-44</t>
+  </si>
+  <si>
+    <t>Update_on_single_filing_system_through_API_based_integration_between_Stock_Excha_40202074.pdf</t>
+  </si>
+  <si>
+    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/Listed Companies/Circular-BSE/2026/February/Update_on_single_filing_system_through_API_based_integration_between_Stock_Excha_40202074.pdf</t>
+  </si>
+  <si>
+    <t>2026-02-03</t>
+  </si>
+  <si>
+    <t>Master Circular for compliance with the provisions of the SEBI (LODR) Regulations, 2015 by listed entities</t>
+  </si>
+  <si>
+    <t>https://www.bseindia.com/markets/MarketInfo/DispNewNoticesCirculars?page=20260203-14</t>
+  </si>
+  <si>
+    <t>Master_Circular_for_compliance_with_the_provisions_of_the_SEBI_LODR_Regulations_06d874e0.pdf</t>
+  </si>
+  <si>
+    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/Listed Companies/Circular-BSE/2026/February/Master_Circular_for_compliance_with_the_provisions_of_the_SEBI_LODR_Regulations_06d874e0.pdf</t>
+  </si>
+  <si>
+    <t>SEBI (Issue and Listing of Non-Convertible Securities)(Amendment) Regulations, 2026</t>
+  </si>
+  <si>
+    <t>https://www.bseindia.com/markets/MarketInfo/DispNewNoticesCirculars?page=20260203-13</t>
+  </si>
+  <si>
+    <t>SEBI_Issue_and_Listing_of_Non_Convertible_Securities_Amendment_Regulations_2026_cc21a9b9.pdf</t>
+  </si>
+  <si>
+    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/Listed Companies/Circular-BSE/2026/February/SEBI_Issue_and_Listing_of_Non_Convertible_Securities_Amendment_Regulations_2026_cc21a9b9.pdf</t>
+  </si>
+  <si>
+    <t>SEBI (Listing Obligations and Disclosure Requirements) (Amendment) Regulations, 2026</t>
+  </si>
+  <si>
+    <t>https://www.bseindia.com/markets/MarketInfo/DispNewNoticesCirculars?page=20260203-12</t>
+  </si>
+  <si>
+    <t>SEBI_Listing_Obligations_and_Disclosure_Requirements_Amendment_Regulations_2026_fff9caaa.pdf</t>
+  </si>
+  <si>
+    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/Listed Companies/Circular-BSE/2026/February/SEBI_Listing_Obligations_and_Disclosure_Requirements_Amendment_Regulations_2026_fff9caaa.pdf</t>
+  </si>
+  <si>
+    <t>2026-02-02</t>
+  </si>
+  <si>
+    <t>Ease of Doing Investment -Special Window for Transfer and Dematerialisation of Physical Securities</t>
+  </si>
+  <si>
+    <t>https://www.bseindia.com/markets/MarketInfo/DispNewNoticesCirculars?page=20260202-37</t>
+  </si>
+  <si>
+    <t>Ease_of_Doing_Investment_Special_Window_for_Transfer_and_Dematerialisation_of_Ph_06eed4b5.pdf</t>
+  </si>
+  <si>
+    <t>/Users/admin/Downloads/Tejomaya_pdfs/Akshayam Data/Listed Companies/Circular-BSE/2026/February/Ease_of_Doing_Investment_Special_Window_for_Transfer_and_Dematerialisation_of_Ph_06eed4b5.pdf</t>
   </si>
 </sst>
 </file>
@@ -174,7 +339,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -199,6 +364,12 @@
       <u/>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -245,7 +416,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -263,6 +434,18 @@
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -576,18 +759,18 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="7" width="114.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="11" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="11" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="11" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="11" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="11" width="114.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="11" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="11" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
@@ -851,16 +1034,346 @@
         <v>50</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="17.25">
+      <c r="A10" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="7">
+        <v>2026</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="17.25">
+      <c r="A11" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="7">
+        <v>2026</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="17.25">
+      <c r="A12" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" s="7">
+        <v>2026</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="17.25">
+      <c r="A13" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="7">
+        <v>2026</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="17.25">
+      <c r="A14" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="7">
+        <v>2026</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25">
+      <c r="A15" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C15" s="9">
+        <v>2026</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25">
+      <c r="A16" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C16" s="9">
+        <v>2026</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="17.25">
+      <c r="A17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C17" s="9">
+        <v>2026</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="17.25">
+      <c r="A18" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C18" s="9">
+        <v>2026</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25">
+      <c r="A19" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C19" s="9">
+        <v>2026</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="17.25">
+      <c r="A20" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C20" s="9">
+        <v>2026</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="G20" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="17.25">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
+      <c r="A22" s="3"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>